<commit_message>
Corrida | SFE-IND | 2026-05-26 12:48:30.202736
</commit_message>
<xml_diff>
--- a/indicadores/SFE-IND_out.xlsx
+++ b/indicadores/SFE-IND_out.xlsx
@@ -107,7 +107,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">28/04/2026</t>
+    <t xml:space="preserve">26/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2156,7 +2156,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.493610590480014</v>
+        <v>0.491431008627311</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2214,7 +2214,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.24079352165545</v>
+        <v>0.239320039908067</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2284,7 +2284,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.000000185626752526868</v>
+        <v>0.00000032167060119318</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2314,7 +2314,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.104045330776329</v>
+        <v>0.138474866962817</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -26903,7 +26903,7 @@
         <v>517</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0281913439416201</v>
+        <v>0.0288840517792924</v>
       </c>
     </row>
     <row r="6">
@@ -26911,7 +26911,7 @@
         <v>518</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0431013014956574</v>
+        <v>0.0454225588775476</v>
       </c>
     </row>
     <row r="7">
@@ -26919,7 +26919,7 @@
         <v>519</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0691279978192014</v>
+        <v>0.0725867598854501</v>
       </c>
     </row>
     <row r="8">
@@ -26927,7 +26927,7 @@
         <v>520</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.112671500499741</v>
+        <v>0.117386885287622</v>
       </c>
     </row>
     <row r="9">
@@ -26935,7 +26935,7 @@
         <v>521</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.179669662932083</v>
+        <v>0.183347231192399</v>
       </c>
     </row>
     <row r="10">
@@ -26943,7 +26943,7 @@
         <v>522</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.261910099887534</v>
+        <v>0.262583981407866</v>
       </c>
     </row>
     <row r="11">
@@ -26951,7 +26951,7 @@
         <v>523</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.347335731705063</v>
+        <v>0.346362724938018</v>
       </c>
     </row>
     <row r="12">
@@ -26959,7 +26959,7 @@
         <v>524</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.432906143077072</v>
+        <v>0.431066995397459</v>
       </c>
     </row>
     <row r="13">
@@ -26967,7 +26967,7 @@
         <v>525</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.493610590480014</v>
+        <v>0.491431008627311</v>
       </c>
     </row>
     <row r="14">
@@ -26975,7 +26975,7 @@
         <v>526</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.49070716487071</v>
+        <v>0.48920347495502</v>
       </c>
     </row>
     <row r="15">
@@ -26983,7 +26983,7 @@
         <v>527</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.41669212559309</v>
+        <v>0.41521945152335</v>
       </c>
     </row>
     <row r="16">
@@ -26991,7 +26991,7 @@
         <v>528</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.308802130064272</v>
+        <v>0.305998409448985</v>
       </c>
     </row>
     <row r="17">
@@ -26999,7 +26999,7 @@
         <v>529</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.216464911933536</v>
+        <v>0.211846895474851</v>
       </c>
     </row>
     <row r="18">
@@ -27007,7 +27007,7 @@
         <v>530</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.150040568594647</v>
+        <v>0.144716200328515</v>
       </c>
     </row>
     <row r="19">
@@ -27015,7 +27015,7 @@
         <v>531</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0909626273358055</v>
+        <v>0.0868630859273947</v>
       </c>
     </row>
     <row r="20">
@@ -27023,7 +27023,7 @@
         <v>532</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0313809702228039</v>
+        <v>0.0288896829026296</v>
       </c>
     </row>
     <row r="21">
@@ -27031,7 +27031,7 @@
         <v>533</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0278045115422365</v>
+        <v>-0.0280627759512987</v>
       </c>
     </row>
     <row r="22">
@@ -27039,7 +27039,7 @@
         <v>534</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0836017885694438</v>
+        <v>-0.0814936598299488</v>
       </c>
     </row>
     <row r="23">
@@ -27047,7 +27047,7 @@
         <v>535</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.13862798825737</v>
+        <v>-0.135914116691038</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-IND | 2026-05-27 10:50:40.96079
</commit_message>
<xml_diff>
--- a/indicadores/SFE-IND_out.xlsx
+++ b/indicadores/SFE-IND_out.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">26/05/2026</t>
+    <t xml:space="preserve">27/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2153,7 +2153,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.49090316893927</v>
+        <v>0.491004097519599</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2211,7 +2211,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.238467067867644</v>
+        <v>0.239392528727023</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2281,7 +2281,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.000000303266903529027</v>
+        <v>0.000000244201402738237</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2311,7 +2311,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.127143560546445</v>
+        <v>0.120216559671304</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -26936,7 +26936,7 @@
         <v>516</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0252310368907169</v>
+        <v>0.0253975048882429</v>
       </c>
     </row>
     <row r="6">
@@ -26944,7 +26944,7 @@
         <v>517</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0442794933421822</v>
+        <v>0.0447601978446472</v>
       </c>
     </row>
     <row r="7">
@@ -26952,7 +26952,7 @@
         <v>518</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0714285999900267</v>
+        <v>0.0724572143388524</v>
       </c>
     </row>
     <row r="8">
@@ -26960,7 +26960,7 @@
         <v>519</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.115592574871119</v>
+        <v>0.117211662773035</v>
       </c>
     </row>
     <row r="9">
@@ -26968,7 +26968,7 @@
         <v>520</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.183768994366327</v>
+        <v>0.18526792125822</v>
       </c>
     </row>
     <row r="10">
@@ -26976,7 +26976,7 @@
         <v>521</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.265653211502649</v>
+        <v>0.26629825724413</v>
       </c>
     </row>
     <row r="11">
@@ -26984,7 +26984,7 @@
         <v>522</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.349112849598459</v>
+        <v>0.348915573462453</v>
       </c>
     </row>
     <row r="12">
@@ -26992,7 +26992,7 @@
         <v>523</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.432104250364803</v>
+        <v>0.431640817711087</v>
       </c>
     </row>
     <row r="13">
@@ -27000,7 +27000,7 @@
         <v>524</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.49090316893927</v>
+        <v>0.491004097519599</v>
       </c>
     </row>
     <row r="14">
@@ -27008,7 +27008,7 @@
         <v>525</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.488330899972184</v>
+        <v>0.489277557963803</v>
       </c>
     </row>
     <row r="15">
@@ -27016,7 +27016,7 @@
         <v>526</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.417005784598332</v>
+        <v>0.418112261464107</v>
       </c>
     </row>
     <row r="16">
@@ -27024,7 +27024,7 @@
         <v>527</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.309556690069763</v>
+        <v>0.310595970063336</v>
       </c>
     </row>
     <row r="17">
@@ -27032,7 +27032,7 @@
         <v>528</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.214109694043333</v>
+        <v>0.215631823306435</v>
       </c>
     </row>
     <row r="18">
@@ -27040,7 +27040,7 @@
         <v>529</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.149111692435005</v>
+        <v>0.150845245806964</v>
       </c>
     </row>
     <row r="19">
@@ -27048,7 +27048,7 @@
         <v>530</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0953200516688361</v>
+        <v>0.0961302714647856</v>
       </c>
     </row>
     <row r="20">
@@ -27056,7 +27056,7 @@
         <v>531</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0378557744304418</v>
+        <v>0.0369996730998714</v>
       </c>
     </row>
     <row r="21">
@@ -27064,7 +27064,7 @@
         <v>532</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0218320856362477</v>
+        <v>-0.0240449639425959</v>
       </c>
     </row>
     <row r="22">
@@ -27072,7 +27072,7 @@
         <v>533</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0793634518932175</v>
+        <v>-0.0818800205106805</v>
       </c>
     </row>
     <row r="23">
@@ -27080,7 +27080,7 @@
         <v>534</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.134565978235849</v>
+        <v>-0.136252429313983</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-IND | 2026-06-17 12:04:10.805196
</commit_message>
<xml_diff>
--- a/indicadores/SFE-IND_out.xlsx
+++ b/indicadores/SFE-IND_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="535">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="537">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Índice Compuesto de Evolución Industrial (ICEI) de la provincia de Santa Fe</t>
+    <t xml:space="preserve">Índice Compuesto de Evolución Industrial (ICEI)</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">27/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2121,9 +2127,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2134,7 +2144,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2148,12 +2158,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.494963664681733</v>
+        <v>0.49411479742429</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2164,7 +2174,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2192,7 +2202,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2206,12 +2216,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.242909822202608</v>
+        <v>0.243189740500479</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2234,7 +2244,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2248,7 +2258,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2262,7 +2272,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2276,12 +2286,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.000000157346684608586</v>
+        <v>0.000000182875822966561</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2292,7 +2302,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2306,12 +2316,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.102002023444872</v>
+        <v>0.0992061279883595</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2454,10 +2464,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2470,10 +2480,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2497,66 +2507,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>96.9973748768791</v>
@@ -2609,7 +2619,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>96.9074470334956</v>
@@ -2666,7 +2676,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>96.9926865753318</v>
@@ -2723,7 +2733,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>97.8645173779358</v>
@@ -2780,7 +2790,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>99.1416966603598</v>
@@ -2837,7 +2847,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>100.267118531735</v>
@@ -2894,7 +2904,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>100.535958864688</v>
@@ -2951,7 +2961,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>100.306763638724</v>
@@ -3008,7 +3018,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>100.712613712781</v>
@@ -3065,7 +3075,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>101.97842526072</v>
@@ -3122,7 +3132,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>103.526803157017</v>
@@ -3179,7 +3189,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>104.768594310333</v>
@@ -3236,7 +3246,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>105.4295567231</v>
@@ -3295,7 +3305,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>105.827101004792</v>
@@ -3354,7 +3364,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>106.376609217875</v>
@@ -3413,7 +3423,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>107.057588987124</v>
@@ -3472,7 +3482,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>107.538951661748</v>
@@ -3531,7 +3541,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>107.632826176099</v>
@@ -3590,7 +3600,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>107.070234107765</v>
@@ -3649,7 +3659,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>106.372752921988</v>
@@ -3708,7 +3718,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>106.369444666172</v>
@@ -3767,7 +3777,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>106.580889295351</v>
@@ -3826,7 +3836,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>107.565563247889</v>
@@ -3885,7 +3895,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>109.286695909081</v>
@@ -3944,7 +3954,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>110.90274460622</v>
@@ -4003,7 +4013,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>112.042362592208</v>
@@ -4062,7 +4072,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>111.877021765825</v>
@@ -4121,7 +4131,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>111.788105051695</v>
@@ -4180,7 +4190,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>112.693660011025</v>
@@ -4239,7 +4249,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>113.442937540792</v>
@@ -4298,7 +4308,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>114.09826254111</v>
@@ -4357,7 +4367,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>114.562728244978</v>
@@ -4416,7 +4426,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>114.601832666931</v>
@@ -4475,7 +4485,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>114.963373120454</v>
@@ -4534,7 +4544,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>115.419254423555</v>
@@ -4593,7 +4603,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>114.759627430106</v>
@@ -4652,7 +4662,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>113.712682870492</v>
@@ -4711,7 +4721,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>114.143360048389</v>
@@ -4770,7 +4780,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>115.297479606145</v>
@@ -4829,7 +4839,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>114.866507102296</v>
@@ -4888,7 +4898,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>113.437636466381</v>
@@ -4947,7 +4957,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>113.295193226658</v>
@@ -5006,7 +5016,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>113.966465307575</v>
@@ -5065,7 +5075,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>114.007609827404</v>
@@ -5124,7 +5134,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>113.419795472036</v>
@@ -5183,7 +5193,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>112.327095276386</v>
@@ -5242,7 +5252,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>110.731538724216</v>
@@ -5301,7 +5311,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>109.9787741636</v>
@@ -5360,7 +5370,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>110.794595296475</v>
@@ -5419,7 +5429,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>112.397156798201</v>
@@ -5478,7 +5488,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>114.455052929728</v>
@@ -5537,7 +5547,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>116.219414403004</v>
@@ -5596,7 +5606,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>116.792767058107</v>
@@ -5655,7 +5665,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>116.839872509861</v>
@@ -5714,7 +5724,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>118.089418727666</v>
@@ -5773,7 +5783,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>120.095105048194</v>
@@ -5832,7 +5842,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>121.424040679636</v>
@@ -5891,7 +5901,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>121.782744591674</v>
@@ -5950,7 +5960,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>121.719627258522</v>
@@ -6009,7 +6019,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>122.192449354742</v>
@@ -6068,7 +6078,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>122.287037092103</v>
@@ -6127,7 +6137,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>120.882488380755</v>
@@ -6186,7 +6196,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>119.882830476384</v>
@@ -6245,7 +6255,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>121.099405181125</v>
@@ -6304,7 +6314,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>122.951264734586</v>
@@ -6363,7 +6373,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>122.828533457862</v>
@@ -6422,7 +6432,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>121.904574093552</v>
@@ -6481,7 +6491,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>122.014910948294</v>
@@ -6540,7 +6550,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>122.728977776998</v>
@@ -6599,7 +6609,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>123.210817095707</v>
@@ -6658,7 +6668,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>122.472815345125</v>
@@ -6717,7 +6727,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>121.948277326746</v>
@@ -6776,7 +6786,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>122.630908940599</v>
@@ -6835,7 +6845,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>122.994805569317</v>
@@ -6894,7 +6904,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>122.888478528227</v>
@@ -6953,7 +6963,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>121.778695987089</v>
@@ -7012,7 +7022,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>120.047275995755</v>
@@ -7071,7 +7081,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>118.829187729906</v>
@@ -7130,7 +7140,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>117.807563715514</v>
@@ -7189,7 +7199,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>117.208797365251</v>
@@ -7248,7 +7258,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>116.806223621756</v>
@@ -7307,7 +7317,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>116.548699832219</v>
@@ -7366,7 +7376,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>117.541936991157</v>
@@ -7425,7 +7435,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>118.152361656455</v>
@@ -7484,7 +7494,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>117.083528213251</v>
@@ -7543,7 +7553,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>115.965131765562</v>
@@ -7602,7 +7612,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>115.658365573433</v>
@@ -7661,7 +7671,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>115.759717022496</v>
@@ -7720,7 +7730,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>115.449623232294</v>
@@ -7779,7 +7789,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>114.526004112896</v>
@@ -7838,7 +7848,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>113.149508061212</v>
@@ -7897,7 +7907,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>111.638451095385</v>
@@ -7956,7 +7966,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>110.33458634863</v>
@@ -8015,7 +8025,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>109.326854099535</v>
@@ -8074,7 +8084,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>108.730458682537</v>
@@ -8133,7 +8143,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>107.645969877825</v>
@@ -8192,7 +8202,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>106.636495071016</v>
@@ -8251,7 +8261,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>107.219436150317</v>
@@ -8310,7 +8320,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>108.897922745878</v>
@@ -8369,7 +8379,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>111.257654500126</v>
@@ -8428,7 +8438,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>113.529710818279</v>
@@ -8487,7 +8497,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>115.229194051517</v>
@@ -8546,7 +8556,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>116.751645600146</v>
@@ -8605,7 +8615,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>117.482194693038</v>
@@ -8664,7 +8674,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>116.986054748093</v>
@@ -8723,7 +8733,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>116.356249564688</v>
@@ -8782,7 +8792,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>116.078179823873</v>
@@ -8841,7 +8851,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>116.318777897703</v>
@@ -8900,7 +8910,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>116.815066609184</v>
@@ -8959,7 +8969,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>116.72637170112</v>
@@ -9018,7 +9028,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>115.988049601792</v>
@@ -9077,7 +9087,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>115.389608960853</v>
@@ -9136,7 +9146,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>116.758313699141</v>
@@ -9195,7 +9205,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>120.093345324775</v>
@@ -9254,7 +9264,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>123.221830053645</v>
@@ -9313,7 +9323,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>125.443891868984</v>
@@ -9372,7 +9382,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>127.79747715177</v>
@@ -9431,7 +9441,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>130.604514444164</v>
@@ -9490,7 +9500,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>132.714690304778</v>
@@ -9549,7 +9559,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>133.831656762021</v>
@@ -9608,7 +9618,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>135.023495877952</v>
@@ -9667,7 +9677,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>136.692115702626</v>
@@ -9726,7 +9736,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>137.031334461638</v>
@@ -9785,7 +9795,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>136.603002592408</v>
@@ -9844,7 +9854,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>136.770994427245</v>
@@ -9903,7 +9913,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>135.559614162002</v>
@@ -9962,7 +9972,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>133.420976735874</v>
@@ -10021,7 +10031,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>132.614651254613</v>
@@ -10080,7 +10090,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>132.659643590571</v>
@@ -10139,7 +10149,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>132.852994998492</v>
@@ -10198,7 +10208,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>133.48819829997</v>
@@ -10257,7 +10267,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>135.102056716535</v>
@@ -10316,7 +10326,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>137.42864647112</v>
@@ -10375,7 +10385,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>139.651943717561</v>
@@ -10434,7 +10444,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>141.084702997884</v>
@@ -10493,7 +10503,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>141.09262135227</v>
@@ -10552,7 +10562,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>140.432544609112</v>
@@ -10611,7 +10621,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>141.227321325612</v>
@@ -10670,7 +10680,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>143.142914524339</v>
@@ -10729,7 +10739,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>144.663942615027</v>
@@ -10788,7 +10798,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>145.986414800313</v>
@@ -10847,7 +10857,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>146.850494342044</v>
@@ -10906,7 +10916,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>147.90405452541</v>
@@ -10965,7 +10975,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>149.095113604505</v>
@@ -11024,7 +11034,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>147.920918220253</v>
@@ -11083,7 +11093,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>145.752803521472</v>
@@ -11142,7 +11152,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>144.848215136569</v>
@@ -11201,7 +11211,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>144.016391574437</v>
@@ -11260,7 +11270,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>144.033677042149</v>
@@ -11319,7 +11329,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>146.286876343536</v>
@@ -11378,7 +11388,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>148.65569405749</v>
@@ -11437,7 +11447,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>149.765460229459</v>
@@ -11496,7 +11506,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>150.131154366799</v>
@@ -11555,7 +11565,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>149.442969761073</v>
@@ -11614,7 +11624,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>147.811366576699</v>
@@ -11673,7 +11683,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>146.72064448369</v>
@@ -11732,7 +11742,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>146.907612856556</v>
@@ -11791,7 +11801,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>147.629112529855</v>
@@ -11850,7 +11860,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>148.02663039464</v>
@@ -11909,7 +11919,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>148.034009722967</v>
@@ -11968,7 +11978,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>148.177062297042</v>
@@ -12027,7 +12037,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>147.612748070027</v>
@@ -12086,7 +12096,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>146.255843034642</v>
@@ -12145,7 +12155,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>146.387547452485</v>
@@ -12204,7 +12214,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>148.527916069814</v>
@@ -12263,7 +12273,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>152.239666213813</v>
@@ -12322,7 +12332,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>155.651469709841</v>
@@ -12381,7 +12391,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>156.611422201364</v>
@@ -12440,7 +12450,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>156.280929927918</v>
@@ -12499,7 +12509,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>155.011999888759</v>
@@ -12558,7 +12568,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>153.184163732435</v>
@@ -12617,7 +12627,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>152.079922394501</v>
@@ -12676,7 +12686,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>151.355845450684</v>
@@ -12735,7 +12745,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>151.382771006582</v>
@@ -12794,7 +12804,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>152.185072555763</v>
@@ -12853,7 +12863,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>152.423745096501</v>
@@ -12912,7 +12922,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>150.933822463028</v>
@@ -12971,7 +12981,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>148.872447679141</v>
@@ -13030,7 +13040,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>147.78514684538</v>
@@ -13089,7 +13099,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>147.084704881082</v>
@@ -13148,7 +13158,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>147.349597486393</v>
@@ -13207,7 +13217,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>147.461676862922</v>
@@ -13266,7 +13276,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>146.3049684633</v>
@@ -13325,7 +13335,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>145.639269523461</v>
@@ -13384,7 +13394,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>144.576681430523</v>
@@ -13443,7 +13453,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>142.763690518045</v>
@@ -13502,7 +13512,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>141.451842586813</v>
@@ -13561,7 +13571,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>139.440836883507</v>
@@ -13620,7 +13630,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>137.937598743733</v>
@@ -13679,7 +13689,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>139.021260380208</v>
@@ -13738,7 +13748,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>140.546866669029</v>
@@ -13797,7 +13807,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>141.849851476618</v>
@@ -13856,7 +13866,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>142.853104458776</v>
@@ -13915,7 +13925,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>143.794642538081</v>
@@ -13974,7 +13984,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>146.26716030859</v>
@@ -14033,7 +14043,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>149.799223894752</v>
@@ -14092,7 +14102,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>152.383921677133</v>
@@ -14151,7 +14161,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>153.186418236673</v>
@@ -14210,7 +14220,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>154.088375186468</v>
@@ -14269,7 +14279,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>155.158423809237</v>
@@ -14328,7 +14338,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>154.592146410844</v>
@@ -14387,7 +14397,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>153.134776185091</v>
@@ -14446,7 +14456,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>151.618985592263</v>
@@ -14505,7 +14515,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>151.059997192368</v>
@@ -14564,7 +14574,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>152.415749334275</v>
@@ -14623,7 +14633,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>154.0259335681</v>
@@ -14682,7 +14692,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>155.488556862998</v>
@@ -14741,7 +14751,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>157.023387453713</v>
@@ -14800,7 +14810,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>156.785079806517</v>
@@ -14859,7 +14869,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>155.399708616518</v>
@@ -14918,7 +14928,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>154.874966708655</v>
@@ -14977,7 +14987,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>156.097333048787</v>
@@ -15036,7 +15046,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>158.326256669047</v>
@@ -15095,7 +15105,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>158.637394575699</v>
@@ -15154,7 +15164,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>158.28026418823</v>
@@ -15213,7 +15223,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>158.516743339679</v>
@@ -15272,7 +15282,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>158.081755685836</v>
@@ -15331,7 +15341,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>157.493259875357</v>
@@ -15390,7 +15400,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>154.97777484048</v>
@@ -15449,7 +15459,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>150.408670516961</v>
@@ -15508,7 +15518,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>147.064418664434</v>
@@ -15567,7 +15577,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>144.671304560147</v>
@@ -15626,7 +15636,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>142.867844348193</v>
@@ -15685,7 +15695,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>143.020338939786</v>
@@ -15744,7 +15754,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>144.257427263235</v>
@@ -15803,7 +15813,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>144.693840724508</v>
@@ -15862,7 +15872,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>144.76644253508</v>
@@ -15921,7 +15931,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>145.425293660953</v>
@@ -15980,7 +15990,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>145.482785438671</v>
@@ -16039,7 +16049,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>145.572138784915</v>
@@ -16098,7 +16108,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>147.98582627173</v>
@@ -16157,7 +16167,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>151.402446790773</v>
@@ -16216,7 +16226,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>153.676709354958</v>
@@ -16275,7 +16285,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>155.361984699416</v>
@@ -16334,7 +16344,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>155.807261985396</v>
@@ -16393,7 +16403,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>154.279815581616</v>
@@ -16452,7 +16462,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>152.426446613539</v>
@@ -16511,7 +16521,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>150.998882372961</v>
@@ -16570,7 +16580,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>149.726179463442</v>
@@ -16629,7 +16639,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>147.924988601437</v>
@@ -16688,7 +16698,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>146.273430577793</v>
@@ -16747,7 +16757,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>146.645025608037</v>
@@ -16806,7 +16816,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>148.384035803093</v>
@@ -16865,7 +16875,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>149.640162205023</v>
@@ -16924,7 +16934,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>150.636592023369</v>
@@ -16983,7 +16993,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>151.33796171197</v>
@@ -17042,7 +17052,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>150.977033686804</v>
@@ -17101,7 +17111,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>150.735599708252</v>
@@ -17160,7 +17170,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>150.731065781381</v>
@@ -17219,7 +17229,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>150.32172690922</v>
@@ -17278,7 +17288,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>149.907392544656</v>
@@ -17337,7 +17347,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>150.024044717991</v>
@@ -17396,7 +17406,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>151.064914395453</v>
@@ -17455,7 +17465,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>150.855903498135</v>
@@ -17514,7 +17524,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>150.465017151074</v>
@@ -17573,7 +17583,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>152.564828238761</v>
@@ -17632,7 +17642,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>155.234708455255</v>
@@ -17691,7 +17701,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>156.797872610488</v>
@@ -17750,7 +17760,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>156.664207307754</v>
@@ -17809,7 +17819,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>156.121040619941</v>
@@ -17868,7 +17878,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>156.101449407873</v>
@@ -17927,7 +17937,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>155.590033615592</v>
@@ -17986,7 +17996,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>154.496259149988</v>
@@ -18045,7 +18055,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>153.587246992414</v>
@@ -18104,7 +18114,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>153.031596025798</v>
@@ -18163,7 +18173,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>152.179182565317</v>
@@ -18222,7 +18232,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>149.806865518511</v>
@@ -18281,7 +18291,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>146.09860032869</v>
@@ -18340,7 +18350,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>143.659377872064</v>
@@ -18399,7 +18409,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>142.704911645731</v>
@@ -18458,7 +18468,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>143.895906760951</v>
@@ -18517,7 +18527,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>146.397507351812</v>
@@ -18576,7 +18586,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>147.248217889281</v>
@@ -18635,7 +18645,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>148.2362022123</v>
@@ -18694,7 +18704,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>150.675460937017</v>
@@ -18753,7 +18763,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>151.14728667222</v>
@@ -18812,7 +18822,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>148.846991090076</v>
@@ -18871,7 +18881,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>147.645318958628</v>
@@ -18930,7 +18940,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>147.780259262999</v>
@@ -18989,7 +18999,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>148.355445566618</v>
@@ -19048,7 +19058,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>148.764787591539</v>
@@ -19107,7 +19117,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>147.511965113582</v>
@@ -19166,7 +19176,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>146.107180872072</v>
@@ -19225,7 +19235,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>145.714316084776</v>
@@ -19284,7 +19294,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>146.586870736786</v>
@@ -19343,7 +19353,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>147.707596112023</v>
@@ -19402,7 +19412,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>148.173059175235</v>
@@ -19461,7 +19471,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>150.03472926627</v>
@@ -19520,7 +19530,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>152.345093909096</v>
@@ -19579,7 +19589,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>153.471079174716</v>
@@ -19638,7 +19648,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>154.090680490467</v>
@@ -19697,7 +19707,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>152.198674795158</v>
@@ -19756,7 +19766,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>148.857979854621</v>
@@ -19815,7 +19825,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>147.224033466198</v>
@@ -19874,7 +19884,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>145.644428003403</v>
@@ -19933,7 +19943,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>143.582668994899</v>
@@ -19992,7 +20002,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>142.913854249233</v>
@@ -20051,7 +20061,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>143.4445085442</v>
@@ -20110,7 +20120,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>143.359968214505</v>
@@ -20169,7 +20179,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>142.883086305977</v>
@@ -20228,7 +20238,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>142.732079729195</v>
@@ -20287,7 +20297,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>142.41658825914</v>
@@ -20346,7 +20356,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>142.457510301466</v>
@@ -20405,7 +20415,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>142.931687634703</v>
@@ -20464,7 +20474,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>144.104825156487</v>
@@ -20523,7 +20533,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>146.52277439968</v>
@@ -20582,7 +20592,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>148.810220634145</v>
@@ -20641,7 +20651,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>150.065016707378</v>
@@ -20700,7 +20710,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>150.888561110485</v>
@@ -20759,7 +20769,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>150.887923162014</v>
@@ -20818,7 +20828,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>148.841401140738</v>
@@ -20877,7 +20887,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>146.146671676579</v>
@@ -20936,7 +20946,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>144.641209679479</v>
@@ -20995,7 +21005,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>143.270448749276</v>
@@ -21054,7 +21064,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>141.140003427095</v>
@@ -21113,7 +21123,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>140.515878511325</v>
@@ -21172,7 +21182,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>141.372562709143</v>
@@ -21231,7 +21241,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>141.765366309835</v>
@@ -21290,7 +21300,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>143.03012753718</v>
@@ -21349,7 +21359,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>145.078953307714</v>
@@ -21408,7 +21418,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>145.353857235894</v>
@@ -21467,7 +21477,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>145.44638111447</v>
@@ -21526,7 +21536,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>147.926800222782</v>
@@ -21585,7 +21595,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>151.020873953677</v>
@@ -21644,7 +21654,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>154.005423195373</v>
@@ -21703,7 +21713,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>156.976009739397</v>
@@ -21762,7 +21772,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>158.828363268872</v>
@@ -21821,7 +21831,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>158.747354838055</v>
@@ -21880,7 +21890,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>157.735672386114</v>
@@ -21939,7 +21949,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>158.446845620188</v>
@@ -21998,7 +22008,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>160.089416073311</v>
@@ -22057,7 +22067,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>160.802112673381</v>
@@ -22116,7 +22126,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>161.569937965902</v>
@@ -22175,7 +22185,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>161.349569437601</v>
@@ -22234,7 +22244,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>160.650452108783</v>
@@ -22293,7 +22303,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>161.137791380292</v>
@@ -22352,7 +22362,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>161.232342877529</v>
@@ -22411,7 +22421,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>161.490526564954</v>
@@ -22470,7 +22480,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>162.584385343726</v>
@@ -22529,7 +22539,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>164.198720644288</v>
@@ -22588,7 +22598,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>165.364858102356</v>
@@ -22647,7 +22657,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>164.417412198747</v>
@@ -22706,7 +22716,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>161.821121481596</v>
@@ -22765,7 +22775,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>159.640955167436</v>
@@ -22824,7 +22834,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>158.576266399433</v>
@@ -22883,7 +22893,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>158.016753301316</v>
@@ -22942,7 +22952,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>158.600102430369</v>
@@ -23001,7 +23011,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>158.54840964767</v>
@@ -23060,7 +23070,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>155.853938851451</v>
@@ -23119,7 +23129,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>153.570499138601</v>
@@ -23178,7 +23188,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>153.370386968175</v>
@@ -23237,7 +23247,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>153.268000906369</v>
@@ -23296,7 +23306,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>152.533709257603</v>
@@ -23355,7 +23365,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>151.414706992451</v>
@@ -23414,7 +23424,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>149.894581927556</v>
@@ -23473,7 +23483,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>147.573621647071</v>
@@ -23532,7 +23542,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>144.667944522659</v>
@@ -23591,7 +23601,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>143.115733805169</v>
@@ -23650,7 +23660,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>142.214661015246</v>
@@ -23709,7 +23719,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>141.727238824975</v>
@@ -23768,7 +23778,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>143.055249392064</v>
@@ -23827,7 +23837,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>144.138481713883</v>
@@ -23886,7 +23896,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>144.58821321343</v>
@@ -23945,7 +23955,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>145.811834737601</v>
@@ -24004,7 +24014,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>147.279243121572</v>
@@ -24063,7 +24073,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>149.136376172176</v>
@@ -24122,7 +24132,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>150.082833202941</v>
@@ -24181,7 +24191,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>149.819082559983</v>
@@ -24240,7 +24250,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>151.252709019271</v>
@@ -24299,7 +24309,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>153.168631384388</v>
@@ -24358,7 +24368,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>154.001852097247</v>
@@ -24417,7 +24427,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>154.891880428711</v>
@@ -24476,7 +24486,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>155.324676520447</v>
@@ -24535,7 +24545,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>153.944068367157</v>
@@ -24594,7 +24604,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>151.519237719348</v>
@@ -24653,7 +24663,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>150.955890736646</v>
@@ -24712,7 +24722,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>151.807716512542</v>
@@ -24771,7 +24781,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>151.600234017736</v>
@@ -24830,7 +24840,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>152.467379839356</v>
@@ -24889,7 +24899,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>155.388326444764</v>
@@ -24948,7 +24958,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>157.180535501302</v>
@@ -25007,7 +25017,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>157.218443433745</v>
@@ -25066,7 +25076,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>156.529211086391</v>
@@ -25125,7 +25135,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>155.393777413036</v>
@@ -25184,7 +25194,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>154.562848570371</v>
@@ -25243,7 +25253,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>155.379263135219</v>
@@ -25302,7 +25312,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>156.000471445839</v>
@@ -25361,7 +25371,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B389" s="2"/>
       <c r="C389" s="3" t="n">
@@ -25394,7 +25404,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3" t="n">
@@ -25427,7 +25437,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3" t="n">
@@ -25460,7 +25470,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3" t="n">
@@ -25493,7 +25503,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3" t="n">
@@ -25526,7 +25536,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3" t="n">
@@ -25559,7 +25569,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3" t="n">
@@ -25592,7 +25602,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3" t="n">
@@ -25625,7 +25635,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3" t="n">
@@ -25658,7 +25668,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3" t="n">
@@ -25691,7 +25701,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3" t="n">
@@ -25724,7 +25734,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3" t="n">
@@ -25757,7 +25767,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3"/>
@@ -25780,7 +25790,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -25803,7 +25813,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -25826,7 +25836,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -25849,7 +25859,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -25872,7 +25882,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -25895,7 +25905,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25918,7 +25928,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -25941,7 +25951,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -25964,7 +25974,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -25987,7 +25997,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -26010,7 +26020,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -26033,7 +26043,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -26056,7 +26066,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -26079,7 +26089,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -26102,7 +26112,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -26125,7 +26135,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -26148,7 +26158,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -26171,7 +26181,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -26194,7 +26204,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -26217,7 +26227,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -26240,7 +26250,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -26263,7 +26273,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -26286,7 +26296,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -26309,7 +26319,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -26332,7 +26342,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -26355,7 +26365,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -26378,7 +26388,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26401,7 +26411,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26424,7 +26434,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26447,7 +26457,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26470,7 +26480,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -26493,7 +26503,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -26516,7 +26526,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -26539,7 +26549,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -26562,7 +26572,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -26585,7 +26595,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -26608,7 +26618,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -26631,7 +26641,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -26654,7 +26664,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -26677,7 +26687,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -26700,7 +26710,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -26723,7 +26733,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -26746,7 +26756,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -26769,7 +26779,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -26803,97 +26813,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
   </sheetData>
@@ -26917,7 +26927,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -26927,160 +26937,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0272854914307451</v>
+        <v>0.0275270201947555</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0474590573153925</v>
+        <v>0.0478990539550082</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0778870969083144</v>
+        <v>0.0781800547569116</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.127203687310688</v>
+        <v>0.127131909527331</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.197014883303598</v>
+        <v>0.196570952465956</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.276131013795426</v>
+        <v>0.275125770399795</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.356238926013666</v>
+        <v>0.354578893446195</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.436687057517002</v>
+        <v>0.434981129797087</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.494963664681733</v>
+        <v>0.49411479742429</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.492858825834141</v>
+        <v>0.493142718186611</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.419018260401896</v>
+        <v>0.420186049866255</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.309278871373596</v>
+        <v>0.311185839201119</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.216100848195577</v>
+        <v>0.21838106554197</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.15159883832482</v>
+        <v>0.153566207090034</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0918547453483833</v>
+        <v>0.0929229970685482</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0275049025415191</v>
+        <v>0.0275738406727949</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0338760341055344</v>
+        <v>-0.0340286817398995</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0874200294139885</v>
+        <v>-0.0868445981916709</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.137359133088409</v>
+        <v>-0.136240796215823</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-IND | 2026-06-23 12:21:45.826729
</commit_message>
<xml_diff>
--- a/indicadores/SFE-IND_out.xlsx
+++ b/indicadores/SFE-IND_out.xlsx
@@ -110,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">17/06/2026</t>
+    <t xml:space="preserve">23/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">focampo</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2143,9 +2143,7 @@
       <c r="J7" s="1"/>
     </row>
     <row r="8">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
+      <c r="A8"/>
       <c r="B8"/>
       <c r="C8"/>
       <c r="D8"/>
@@ -2157,14 +2155,10 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
+      <c r="A9"/>
       <c r="B9"/>
       <c r="C9"/>
-      <c r="D9" t="n">
-        <v>0.49411479742429</v>
-      </c>
+      <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
       <c r="G9"/>
@@ -2174,13 +2168,11 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
-      <c r="D10" t="n">
-        <v>-1</v>
-      </c>
+      <c r="D10"/>
       <c r="E10"/>
       <c r="F10"/>
       <c r="G10"/>
@@ -2189,10 +2181,14 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11">
-      <c r="A11"/>
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
       <c r="B11"/>
       <c r="C11"/>
-      <c r="D11"/>
+      <c r="D11" t="n">
+        <v>0.495761254179018</v>
+      </c>
       <c r="E11"/>
       <c r="F11"/>
       <c r="G11"/>
@@ -2202,11 +2198,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
-      <c r="D12"/>
+      <c r="D12" t="n">
+        <v>-1</v>
+      </c>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
@@ -2215,14 +2213,10 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
+      <c r="A13"/>
       <c r="B13"/>
       <c r="C13"/>
-      <c r="D13" t="n">
-        <v>0.243189740500479</v>
-      </c>
+      <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
@@ -2231,7 +2225,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14">
-      <c r="A14"/>
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
       <c r="B14"/>
       <c r="C14"/>
       <c r="D14"/>
@@ -2244,11 +2240,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
-      <c r="D15"/>
+      <c r="D15" t="n">
+        <v>0.242536832796444</v>
+      </c>
       <c r="E15"/>
       <c r="F15"/>
       <c r="G15"/>
@@ -2257,9 +2255,7 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16">
-      <c r="A16" t="s">
-        <v>26</v>
-      </c>
+      <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
@@ -2272,7 +2268,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2286,13 +2282,11 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
-      <c r="D18" t="n">
-        <v>0.000000182875822966561</v>
-      </c>
+      <c r="D18"/>
       <c r="E18"/>
       <c r="F18"/>
       <c r="G18"/>
@@ -2302,7 +2296,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2321,7 +2315,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0992061279883595</v>
+        <v>0.0000000852800512903576</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2331,7 +2325,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
       <c r="B21"/>
       <c r="C21"/>
       <c r="D21"/>
@@ -2343,10 +2339,14 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22">
-      <c r="A22"/>
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
       <c r="B22"/>
       <c r="C22"/>
-      <c r="D22"/>
+      <c r="D22" t="n">
+        <v>0.11922867700706</v>
+      </c>
       <c r="E22"/>
       <c r="F22"/>
       <c r="G22"/>
@@ -26946,7 +26946,7 @@
         <v>518</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0275270201947555</v>
+        <v>0.0212937466201707</v>
       </c>
     </row>
     <row r="6">
@@ -26954,7 +26954,7 @@
         <v>519</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0478990539550082</v>
+        <v>0.0403014307890175</v>
       </c>
     </row>
     <row r="7">
@@ -26962,7 +26962,7 @@
         <v>520</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0781800547569116</v>
+        <v>0.0691158949522463</v>
       </c>
     </row>
     <row r="8">
@@ -26970,7 +26970,7 @@
         <v>521</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.127131909527331</v>
+        <v>0.115504239504155</v>
       </c>
     </row>
     <row r="9">
@@ -26978,7 +26978,7 @@
         <v>522</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.196570952465956</v>
+        <v>0.18649211685404</v>
       </c>
     </row>
     <row r="10">
@@ -26986,7 +26986,7 @@
         <v>523</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.275125770399795</v>
+        <v>0.271140528311075</v>
       </c>
     </row>
     <row r="11">
@@ -26994,7 +26994,7 @@
         <v>524</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.354578893446195</v>
+        <v>0.355101574897808</v>
       </c>
     </row>
     <row r="12">
@@ -27002,7 +27002,7 @@
         <v>525</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.434981129797087</v>
+        <v>0.437008454699267</v>
       </c>
     </row>
     <row r="13">
@@ -27010,7 +27010,7 @@
         <v>526</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.49411479742429</v>
+        <v>0.495761254179018</v>
       </c>
     </row>
     <row r="14">
@@ -27018,7 +27018,7 @@
         <v>527</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.493142718186611</v>
+        <v>0.492480286708457</v>
       </c>
     </row>
     <row r="15">
@@ -27026,7 +27026,7 @@
         <v>528</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.420186049866255</v>
+        <v>0.418556431784141</v>
       </c>
     </row>
     <row r="16">
@@ -27034,7 +27034,7 @@
         <v>529</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.311185839201119</v>
+        <v>0.312315148421689</v>
       </c>
     </row>
     <row r="17">
@@ -27042,7 +27042,7 @@
         <v>530</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.21838106554197</v>
+        <v>0.221353043293413</v>
       </c>
     </row>
     <row r="18">
@@ -27050,7 +27050,7 @@
         <v>531</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.153566207090034</v>
+        <v>0.154382501450509</v>
       </c>
     </row>
     <row r="19">
@@ -27058,7 +27058,7 @@
         <v>532</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0929229970685482</v>
+        <v>0.0930179190755681</v>
       </c>
     </row>
     <row r="20">
@@ -27066,7 +27066,7 @@
         <v>533</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0275738406727949</v>
+        <v>0.0298781407731508</v>
       </c>
     </row>
     <row r="21">
@@ -27074,7 +27074,7 @@
         <v>534</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0340286817398995</v>
+        <v>-0.0324162234981954</v>
       </c>
     </row>
     <row r="22">
@@ -27082,7 +27082,7 @@
         <v>535</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0868445981916709</v>
+        <v>-0.0878118879964002</v>
       </c>
     </row>
     <row r="23">
@@ -27090,7 +27090,7 @@
         <v>536</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.136240796215823</v>
+        <v>-0.136591455149325</v>
       </c>
     </row>
     <row r="24">
@@ -27118,4 +27118,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{890674ED-A2E2-4904-8907-A544C76FF4FD}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B39D867-FD83-48EF-A4AA-8FDC43E7E443}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E25A1AB1-7A35-47F3-A750-E5AFCD042170}"/>
 </file>
</xml_diff>